<commit_message>
Record confirmed Premium pricing and task reward multiplier rules
</commit_message>
<xml_diff>
--- a/docs/arkusze/HARBORLIGHT3-zasady.xlsx
+++ b/docs/arkusze/HARBORLIGHT3-zasady.xlsx
@@ -10268,8 +10268,10 @@
       <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>1</v>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Wersja 3 uwzględnia wpisy i trzy kolejne potwierdzenia z 22.10.2026. Zatwierdzono niepełne kursy, proporcjonalną wycenę materiałów Premium oraz utrwalanie mnożnika zadania po kliknięciu. Pozostałe modele i otwarte szczegóły oznaczono osobno. Dokument nie zmienia kodu gry.</t>
+        </is>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -10739,28 +10741,38 @@
       <c r="C15" s="6" t="s">
         <v>630</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>631</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>632</v>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Wiek przy pierwszym kliknięciu: &lt;15 s → ×3; 15 s ≤ wiek &lt;300 s → ×2; od 300 s → ×1.</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Potwierdzone: ×3 ma pierwszeństwo, nie mnoży się przez ×2. Mnożnik zapisuje pierwsze kliknięcie zadania.</t>
+        </is>
       </c>
     </row>
     <row r="16" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
         <v>633</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>598</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>634</v>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>POTWIERDZONE</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Pierwsze kliknięcie konkretnego zadania zapisuje mnożnik aż do jego ukończenia; późniejszy upływ czasu nie zmniejsza zapisanego mnożnika.</t>
+        </is>
       </c>
       <c r="D16" s="5" t="s">
         <v>635</v>
       </c>
-      <c r="E16" s="5" t="s">
-        <v>636</v>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Nagroda dopiero po wpłaceniu całości przed upływem 6 h od pojawienia się zadania. Samo kliknięcie nie wypłaca nagrody. Nieukończenie w terminie oznacza utratę wpłat.</t>
+        </is>
       </c>
     </row>
     <row r="17" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12198,8 +12210,10 @@
       <c r="K1" s="9"/>
     </row>
     <row r="2" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>731</v>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Statyczne przykłady w chwili pierwszego kliknięcia. Kolumna B to wiek w tej chwili, C — czas pozostały w chwili kliknięcia, D — utrwalony mnożnik: &lt;15 s ×3; 15–&lt;300 s ×2; od 300 s ×1. Późniejszy upływ czasu nie przelicza D. Nagroda wymaga pełnej wpłaty przed upływem 6 h. Wszystkie te reguły potwierdzono.</t>
+        </is>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -12229,14 +12243,20 @@
       <c r="A5" s="4" t="s">
         <v>470</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>732</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>439</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>733</v>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Wiek przy pierwszym kliknięciu [s]</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Pozostało w chwili kliknięcia [min]</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Utrwalony mnożnik</t>
+        </is>
       </c>
       <c r="E5" s="4" t="s">
         <v>734</v>
@@ -22729,8 +22749,10 @@
       <c r="E43" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="F43" s="6" t="s">
-        <v>1077</v>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>Potwierdzone: 10 monet za każdy potrzebny kurs, również ostatni niepełny; 100 przy ładunku 60 kosztuje 20 monet.</t>
+        </is>
       </c>
     </row>
     <row r="44" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22749,8 +22771,10 @@
       <c r="E44" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="F44" s="5" t="s">
-        <v>1080</v>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Potwierdzone: proporcjonalne bazowe ceny zakupu portowego; +25% wyłącznie materiałów. Koszt monet budynku doliczany osobno. Bez paczek po 100 w tej wycenie.</t>
+        </is>
       </c>
     </row>
     <row r="45" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22789,8 +22813,10 @@
       <c r="E46" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="F46" s="5" t="s">
-        <v>1087</v>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>Pierwsze kliknięcie konkretnego zadania utrwala ×3 przed upływem 15 s; nagroda po pełnej wpłacie przed końcem 6 h. Potwierdzone.</t>
+        </is>
       </c>
     </row>
     <row r="47" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22809,8 +22835,10 @@
       <c r="E47" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="F47" s="6" t="s">
-        <v>1091</v>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>Od 15 s do przed upływem 5 min pierwsze kliknięcie utrwala ×2; od 5 min ×1. Mnożniki nie sumują się. Potwierdzone.</t>
+        </is>
       </c>
     </row>
     <row r="48" customFormat="false" ht="64.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22934,8 +22962,10 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
-        <v>62</v>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>BUDYNKI V3 • uwzględnione wpisy i potwierdzenia</t>
+        </is>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -23063,8 +23093,10 @@
       <c r="I6" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="J6" s="5" t="s">
-        <v>87</v>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>V3: skrócenie budowy o 25/50/75% — 1 moneta za pełną zaoszczędzoną minutę. Zakup materiałów: proporcjonalna bazowa cena portowa ×1,25, bez paczek po 100; wymagane monety osobno, bez dopłaty 25%. Opłata za skrócenie czasu jest osobna. Podstawa czasu i zaokrąglenie końcowej ceny pozostają modelami. Cena natychmiastowego skrócenia o 100% nie została ustalona.</t>
+        </is>
       </c>
       <c r="K6" s="5" t="s">
         <v>88</v>
@@ -23113,8 +23145,10 @@
       <c r="I7" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="J7" s="6" t="s">
-        <v>87</v>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>V3: skrócenie budowy o 25/50/75% — 1 moneta za pełną zaoszczędzoną minutę. Zakup materiałów: proporcjonalna bazowa cena portowa ×1,25, bez paczek po 100; wymagane monety osobno, bez dopłaty 25%. Opłata za skrócenie czasu jest osobna. Podstawa czasu i zaokrąglenie końcowej ceny pozostają modelami. Cena natychmiastowego skrócenia o 100% nie została ustalona.</t>
+        </is>
       </c>
       <c r="K7" s="6" t="s">
         <v>95</v>
@@ -23163,8 +23197,10 @@
       <c r="I8" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="J8" s="5" t="s">
-        <v>104</v>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>V3: skrócenie budowy o 25/50/75% — 1 moneta za pełną zaoszczędzoną minutę. Zakup materiałów: proporcjonalna bazowa cena portowa ×1,25, bez paczek po 100; wymagane monety osobno, bez dopłaty 25%. Opłata za skrócenie czasu jest osobna. Podstawa czasu i zaokrąglenie końcowej ceny pozostają modelami. Cena natychmiastowego skrócenia o 100% nie została ustalona. Transport Premium: 10 monet za każdy potrzebny kurs, również ostatni niepełny.</t>
+        </is>
       </c>
       <c r="K8" s="5" t="s">
         <v>105</v>
@@ -23213,8 +23249,10 @@
       <c r="I9" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="J9" s="6" t="s">
-        <v>104</v>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>V3: skrócenie budowy o 25/50/75% — 1 moneta za pełną zaoszczędzoną minutę. Zakup materiałów: proporcjonalna bazowa cena portowa ×1,25, bez paczek po 100; wymagane monety osobno, bez dopłaty 25%. Opłata za skrócenie czasu jest osobna. Podstawa czasu i zaokrąglenie końcowej ceny pozostają modelami. Cena natychmiastowego skrócenia o 100% nie została ustalona. Transport Premium: 10 monet za każdy potrzebny kurs, również ostatni niepełny.</t>
+        </is>
       </c>
       <c r="K9" s="6"/>
       <c r="L9" s="6" t="s">
@@ -23261,8 +23299,10 @@
       <c r="I10" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="J10" s="5" t="s">
-        <v>104</v>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>V3: skrócenie budowy o 25/50/75% — 1 moneta za pełną zaoszczędzoną minutę. Zakup materiałów: proporcjonalna bazowa cena portowa ×1,25, bez paczek po 100; wymagane monety osobno, bez dopłaty 25%. Opłata za skrócenie czasu jest osobna. Podstawa czasu i zaokrąglenie końcowej ceny pozostają modelami. Cena natychmiastowego skrócenia o 100% nie została ustalona. Transport Premium: 10 monet za każdy potrzebny kurs, również ostatni niepełny.</t>
+        </is>
       </c>
       <c r="K10" s="5"/>
       <c r="L10" s="5" t="s">
@@ -23309,8 +23349,10 @@
       <c r="I11" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="J11" s="6" t="s">
-        <v>104</v>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>V3: skrócenie budowy o 25/50/75% — 1 moneta za pełną zaoszczędzoną minutę. Zakup materiałów: proporcjonalna bazowa cena portowa ×1,25, bez paczek po 100; wymagane monety osobno, bez dopłaty 25%. Opłata za skrócenie czasu jest osobna. Podstawa czasu i zaokrąglenie końcowej ceny pozostają modelami. Cena natychmiastowego skrócenia o 100% nie została ustalona. Transport Premium: 10 monet za każdy potrzebny kurs, również ostatni niepełny.</t>
+        </is>
       </c>
       <c r="K11" s="6"/>
       <c r="L11" s="6" t="s">
@@ -23357,8 +23399,10 @@
       <c r="I12" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="J12" s="5" t="s">
-        <v>104</v>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>V3: skrócenie budowy o 25/50/75% — 1 moneta za pełną zaoszczędzoną minutę. Zakup materiałów: proporcjonalna bazowa cena portowa ×1,25, bez paczek po 100; wymagane monety osobno, bez dopłaty 25%. Opłata za skrócenie czasu jest osobna. Podstawa czasu i zaokrąglenie końcowej ceny pozostają modelami. Cena natychmiastowego skrócenia o 100% nie została ustalona. Transport Premium: 10 monet za każdy potrzebny kurs, również ostatni niepełny.</t>
+        </is>
       </c>
       <c r="K12" s="5"/>
       <c r="L12" s="5" t="s">
@@ -23405,8 +23449,10 @@
       <c r="I13" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="J13" s="6" t="s">
-        <v>104</v>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>V3: skrócenie budowy o 25/50/75% — 1 moneta za pełną zaoszczędzoną minutę. Zakup materiałów: proporcjonalna bazowa cena portowa ×1,25, bez paczek po 100; wymagane monety osobno, bez dopłaty 25%. Opłata za skrócenie czasu jest osobna. Podstawa czasu i zaokrąglenie końcowej ceny pozostają modelami. Cena natychmiastowego skrócenia o 100% nie została ustalona. Transport Premium: 10 monet za każdy potrzebny kurs, również ostatni niepełny.</t>
+        </is>
       </c>
       <c r="K13" s="6" t="s">
         <v>128</v>
@@ -23455,8 +23501,10 @@
       <c r="I14" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="J14" s="5" t="s">
-        <v>104</v>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>V3: skrócenie budowy o 25/50/75% — 1 moneta za pełną zaoszczędzoną minutę. Zakup materiałów: proporcjonalna bazowa cena portowa ×1,25, bez paczek po 100; wymagane monety osobno, bez dopłaty 25%. Opłata za skrócenie czasu jest osobna. Podstawa czasu i zaokrąglenie końcowej ceny pozostają modelami. Cena natychmiastowego skrócenia o 100% nie została ustalona. Transport Premium: 10 monet za każdy potrzebny kurs, również ostatni niepełny.</t>
+        </is>
       </c>
       <c r="K14" s="5" t="s">
         <v>133</v>
@@ -23505,8 +23553,10 @@
       <c r="I15" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="J15" s="6" t="s">
-        <v>104</v>
+      <c r="J15" s="6" t="inlineStr">
+        <is>
+          <t>V3: skrócenie budowy o 25/50/75% — 1 moneta za pełną zaoszczędzoną minutę. Zakup materiałów: proporcjonalna bazowa cena portowa ×1,25, bez paczek po 100; wymagane monety osobno, bez dopłaty 25%. Opłata za skrócenie czasu jest osobna. Podstawa czasu i zaokrąglenie końcowej ceny pozostają modelami. Cena natychmiastowego skrócenia o 100% nie została ustalona. Transport Premium: 10 monet za każdy potrzebny kurs, również ostatni niepełny.</t>
+        </is>
       </c>
       <c r="K15" s="6" t="s">
         <v>139</v>
@@ -23555,8 +23605,10 @@
       <c r="I16" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="J16" s="5" t="s">
-        <v>87</v>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>V3: skrócenie budowy o 25/50/75% — 1 moneta za pełną zaoszczędzoną minutę. Zakup materiałów: proporcjonalna bazowa cena portowa ×1,25, bez paczek po 100; wymagane monety osobno, bez dopłaty 25%. Opłata za skrócenie czasu jest osobna. Podstawa czasu i zaokrąglenie końcowej ceny pozostają modelami. Cena natychmiastowego skrócenia o 100% nie została ustalona.</t>
+        </is>
       </c>
       <c r="K16" s="5"/>
       <c r="L16" s="5" t="s">
@@ -23603,8 +23655,10 @@
       <c r="I17" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="J17" s="6" t="s">
-        <v>87</v>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>V3: skrócenie budowy o 25/50/75% — 1 moneta za pełną zaoszczędzoną minutę. Zakup materiałów: proporcjonalna bazowa cena portowa ×1,25, bez paczek po 100; wymagane monety osobno, bez dopłaty 25%. Opłata za skrócenie czasu jest osobna. Podstawa czasu i zaokrąglenie końcowej ceny pozostają modelami. Cena natychmiastowego skrócenia o 100% nie została ustalona.</t>
+        </is>
       </c>
       <c r="K17" s="6" t="s">
         <v>157</v>
@@ -24040,51 +24094,69 @@
       <c r="A23" s="6" t="s">
         <v>1176</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>1163</v>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>ROZSTRZYGNIĘTE</t>
+        </is>
       </c>
       <c r="C23" s="6" t="s">
         <v>1177</v>
       </c>
-      <c r="D23" s="6" t="s">
-        <v>1178</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>1179</v>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Liczymy każdy potrzebny kurs, również ostatni niepełny. 100 sztuk / 60 na kurs = 2 kursy = 20 monet.</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Potwierdzenie użytkownika: „Tak, również ostatni niepełny kurs”.</t>
+        </is>
       </c>
     </row>
     <row r="24" customFormat="false" ht="99.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
         <v>1180</v>
       </c>
-      <c r="B24" s="5" t="s">
-        <v>1163</v>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>CZĘŚCIOWO ROZSTRZYGNIĘTE</t>
+        </is>
       </c>
       <c r="C24" s="5" t="s">
         <v>1181</v>
       </c>
-      <c r="D24" s="5" t="s">
-        <v>1182</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>1183</v>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Proporcjonalne bazowe ceny zakupu portowego, bez paczek po 100; materiały +25%, monety osobno.</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Potwierdzone. Do decyzji nadal: cały koszt czy tylko brakujące materiały oraz zaokrąglenie końcowej ceny. Zwykły handel portowy nadal działa w paczkach po 100.</t>
+        </is>
       </c>
     </row>
     <row r="25" customFormat="false" ht="99.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
         <v>1184</v>
       </c>
-      <c r="B25" s="6" t="s">
-        <v>1163</v>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>ROZSTRZYGNIĘTE</t>
+        </is>
       </c>
       <c r="C25" s="6" t="s">
         <v>1185</v>
       </c>
-      <c r="D25" s="6" t="s">
-        <v>1186</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>1187</v>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Wymagane monety budynku doliczamy nominalnie, osobno od materiałów i poza dopłatą 25%.</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Potwierdzenie użytkownika: „Tak, cena proporcjonalna materiałów +25%, monety osobno”.</t>
+        </is>
       </c>
     </row>
     <row r="26" customFormat="false" ht="99.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -24227,17 +24299,23 @@
       <c r="A34" s="5" t="s">
         <v>1221</v>
       </c>
-      <c r="B34" s="5" t="s">
-        <v>1209</v>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>ROZSTRZYGNIĘTE</t>
+        </is>
       </c>
       <c r="C34" s="5" t="s">
         <v>1222</v>
       </c>
-      <c r="D34" s="5" t="s">
-        <v>1223</v>
-      </c>
-      <c r="E34" s="5" t="s">
-        <v>1224</v>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Pierwsze kliknięcie zadania utrwala ×3 przed 15 s, następnie ×2 przed 5 min; od 5 min ×1.</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Potwierdzone: nagroda po pełnej wpłacie przed upływem 6 h. Późniejsze kliknięcia nie podwyższają ani nie obniżają zapisanego mnożnika.</t>
+        </is>
       </c>
     </row>
     <row r="35" customFormat="false" ht="99.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27118,14 +27196,18 @@
       <c r="C142" s="5" t="s">
         <v>1751</v>
       </c>
-      <c r="D142" s="5" t="s">
-        <v>365</v>
+      <c r="D142" s="5" t="inlineStr">
+        <is>
+          <t>POTWIERDZONE</t>
+        </is>
       </c>
       <c r="E142" s="5" t="s">
         <v>1770</v>
       </c>
-      <c r="F142" s="5" t="s">
-        <v>1771</v>
+      <c r="F142" s="5" t="inlineStr">
+        <is>
+          <t>Potwierdzono: ROUNDUP(ilość / ładunek); każdy potrzebny kurs, również ostatni niepełny, kosztuje 10 monet. 100 / 60 wymaga 2 kursów i kosztuje 20 monet. Źródło: odpowiedź użytkownika 22.10.2026.</t>
+        </is>
       </c>
     </row>
     <row r="143" customFormat="false" ht="114.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27198,14 +27280,20 @@
       <c r="C146" s="5" t="s">
         <v>1751</v>
       </c>
-      <c r="D146" s="5" t="s">
-        <v>383</v>
-      </c>
-      <c r="E146" s="5" t="s">
-        <v>1781</v>
-      </c>
-      <c r="F146" s="5" t="s">
-        <v>1782</v>
+      <c r="D146" s="5" t="inlineStr">
+        <is>
+          <t>WYCENA POTWIERDZONA; ZAKRES MATERIAŁÓW OTWARTY</t>
+        </is>
+      </c>
+      <c r="E146" s="5" t="inlineStr">
+        <is>
+          <t>Cena = 1,25 × proporcjonalna bazowa portowa wartość materiałów + wymagane monety budynku + opłata za skrócenie czasu.</t>
+        </is>
+      </c>
+      <c r="F146" s="5" t="inlineStr">
+        <is>
+          <t>Potwierdzone: bez paczek po 100, bazowe ceny zakupu, +25% tylko od materiałów. Pełny koszt czy brakujące materiały i końcowe zaokrąglenie pozostają do decyzji. Źródło: odpowiedź użytkownika 22.10.2026.</t>
+        </is>
       </c>
     </row>
     <row r="147" customFormat="false" ht="114.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27218,14 +27306,20 @@
       <c r="C147" s="6" t="s">
         <v>1751</v>
       </c>
-      <c r="D147" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="E147" s="6" t="s">
-        <v>1784</v>
-      </c>
-      <c r="F147" s="6" t="s">
-        <v>1785</v>
+      <c r="D147" s="6" t="inlineStr">
+        <is>
+          <t>POTWIERDZONE</t>
+        </is>
+      </c>
+      <c r="E147" s="6" t="inlineStr">
+        <is>
+          <t>Monety zapisane w koszcie budynku doliczamy osobno w wymaganej wysokości; nie obejmuje ich dopłata 25%.</t>
+        </is>
+      </c>
+      <c r="F147" s="6" t="inlineStr">
+        <is>
+          <t>Potwierdzenie użytkownika: „Tak, cena proporcjonalna materiałów +25%, monety osobno”.</t>
+        </is>
       </c>
     </row>
     <row r="148" customFormat="false" ht="114.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27561,11 +27655,15 @@
       <c r="D164" s="5" t="s">
         <v>232</v>
       </c>
-      <c r="E164" s="5" t="s">
-        <v>1838</v>
-      </c>
-      <c r="F164" s="5" t="s">
-        <v>1839</v>
+      <c r="E164" s="5" t="inlineStr">
+        <is>
+          <t>Pierwsze kliknięcie: przed upływem 15 s utrwala ×3; od 15 s do przed upływem 300 s utrwala ×2; od 300 s ×1.</t>
+        </is>
+      </c>
+      <c r="F164" s="5" t="inlineStr">
+        <is>
+          <t>Potwierdzone granice i utrwalenie mnożnika; ×3 i ×2 nie mnożą się ze sobą. Źródło: odpowiedź użytkownika 22.10.2026.</t>
+        </is>
       </c>
     </row>
     <row r="165" customFormat="false" ht="114.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27578,14 +27676,20 @@
       <c r="C165" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="D165" s="6" t="s">
-        <v>598</v>
-      </c>
-      <c r="E165" s="6" t="s">
-        <v>1841</v>
-      </c>
-      <c r="F165" s="6" t="s">
-        <v>1842</v>
+      <c r="D165" s="6" t="inlineStr">
+        <is>
+          <t>POTWIERDZONE</t>
+        </is>
+      </c>
+      <c r="E165" s="6" t="inlineStr">
+        <is>
+          <t>Pierwsze kliknięcie konkretnego zadania utrwala mnożnik do ukończenia. Nagroda = bazowa nagroda × utrwalony mnożnik.</t>
+        </is>
+      </c>
+      <c r="F165" s="6" t="inlineStr">
+        <is>
+          <t>Wypłata dopiero po wpłaceniu całości przed upływem 6 h od pojawienia się; samo kliknięcie nie daje nagrody. Źródło: odpowiedź użytkownika 22.10.2026.</t>
+        </is>
       </c>
     </row>
     <row r="166" customFormat="false" ht="114.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29008,14 +29112,20 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="99.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
-        <v>1961</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>1962</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>1963</v>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Potwierdzenia V3</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Zatwierdzono: ostatni niepełny kurs jest płatny; materiały proporcjonalnie według bazowych cen portowych +25%, monety osobno; pierwsze kliknięcie utrwala bonus zadania.</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Odpowiedzi użytkownika 22.10.2026: „Tak, również ostatni niepełny kurs”; „Tak, cena proporcjonalna materiałów +25%, monety osobno”; „Tak, kliknięcie zapisuje mnożnik”. Nagroda za pełną wpłatę przed końcem 6 h. Te trzy pytania są zamknięte; inne szczegóły pozostają oznaczone osobno.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -32041,11 +32151,15 @@
       <c r="C12" s="5" t="s">
         <v>363</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>364</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>365</v>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Potwierdzone: kursy = ROUNDUP(ilość / ładunek, 0). Ostatni niepełny kurs jest płatny. Dla 100 sztuk i ładunku 60 potrzeba 2 kursów, więc cena wynosi 20 monet.</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>POTWIERDZONE</t>
+        </is>
       </c>
     </row>
     <row r="13" customFormat="false" ht="99.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -32103,34 +32217,50 @@
       <c r="A16" s="5" t="s">
         <v>379</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>380</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>381</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>383</v>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Proporcjonalna bazowa cena zakupu materiałów w porcie ×1,25, plus nominalny koszt monet budynku oraz opłata za skrócenie czasu.</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Cena = 1,25 × bazowa portowa wartość materiałów + monety wymagane przez budynek + opłata czasowa.</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Potwierdzone: bez zaokrąglania materiałów do paczek po 100; używamy bazowych cen zakupu, a dopłata 25% obejmuje tylko materiały. Do ustalenia pozostaje pełny koszt czy tylko brakujące materiały oraz końcowe zaokrąglenie ceny.</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>WYCENA POTWIERDZONA; ZAKRES MATERIAŁÓW DO USTALENIA</t>
+        </is>
       </c>
     </row>
     <row r="17" customFormat="false" ht="99.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>385</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>386</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>387</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>388</v>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Monety zapisane w koszcie budynku doliczamy osobno w wymaganej wysokości.</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Wymagane monety + 1,25 × portowa wartość pięciu materiałów; opłata czasowa osobno.</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Potwierdzone: monety nie są materiałem kupowanym w porcie i nie podlegają dopłacie 25%.</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>POTWIERDZONE</t>
+        </is>
       </c>
     </row>
     <row r="18" customFormat="false" ht="99.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -32846,8 +32976,10 @@
       <c r="K1" s="9"/>
     </row>
     <row r="2" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>444</v>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Potwierdzone: każdy potrzebny kurs jest płatny, również ostatni niepełny. Cena = SUMA(ROUNDUP(ilość rodzaju / ładunek)) × liczba odcinków × 10 monet. Dwa rodzaje nie dzielą kursu. Liczba pracowników zmienia czas, a nie liczbę płatnych kursów. Zakres jednego kliknięcia i etapu port–statek pozostaje otwarty.</t>
+        </is>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -33469,8 +33601,10 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="9" t="s">
-        <v>468</v>
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>BUDYNEK PREMIUM • potwierdzona wycena materiałów</t>
+        </is>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -33490,8 +33624,10 @@
       <c r="Q1" s="9"/>
     </row>
     <row r="2" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>469</v>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Potwierdzone: bazowe ceny zakupu portowego liczymy proporcjonalnie do ilości, bez paczek po 100. Materiały ×1,25; wymagane monety nominalnie osobno; opłata czasowa osobno. N/P to aktualny wariant. I/O zachowano jako odrzucone porównanie. Zaokrąglenie końcowej ceny w górę i zakres skracanego czasu pozostają założeniami kalkulatora.</t>
+        </is>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -33551,14 +33687,20 @@
       <c r="G5" s="4" t="s">
         <v>476</v>
       </c>
-      <c r="H5" s="4" t="s">
-        <v>477</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>478</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>479</v>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Port: wycena proporcjonalna — aktualna</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Paczki 100 — wariant odrzucony</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Materiały +25% — zatwierdzone</t>
+        </is>
       </c>
       <c r="K5" s="4" t="s">
         <v>436</v>
@@ -33569,14 +33711,20 @@
       <c r="M5" s="4" t="s">
         <v>480</v>
       </c>
-      <c r="N5" s="4" t="s">
-        <v>481</v>
-      </c>
-      <c r="O5" s="4" t="s">
-        <v>482</v>
-      </c>
-      <c r="P5" s="4" t="s">
-        <v>483</v>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>Razem — aktualna wycena</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>Razem — odrzucone paczki 100</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="inlineStr">
+        <is>
+          <t>PLN — aktualna wycena</t>
+        </is>
       </c>
       <c r="Q5" s="4" t="s">
         <v>332</v>
@@ -33638,8 +33786,10 @@
         <f aca="false">N6/Parametry!$C$41</f>
         <v>31</v>
       </c>
-      <c r="Q6" s="5" t="s">
-        <v>485</v>
+      <c r="Q6" s="5" t="inlineStr">
+        <is>
+          <t>Potwierdzona wycena: 100 drewna = 50 monet, 100 Food = 150; materiały z dopłatą = 250. Przykładowe skrócenie 120 min o 50% kosztuje 60 monet, razem 310. Zakres czasu i końcowe zaokrąglenie nie zostały osobno zatwierdzone.</t>
+        </is>
       </c>
     </row>
     <row r="7" customFormat="false" ht="114.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33699,8 +33849,10 @@
         <f aca="false">N7/Parametry!$C$41</f>
         <v>16.7</v>
       </c>
-      <c r="Q7" s="6" t="s">
-        <v>487</v>
+      <c r="Q7" s="6" t="inlineStr">
+        <is>
+          <t>Farma 1→2: materiały według cen proporcjonalnych z dopłatą kosztują 165 monet. Przykładowa faza budowy 5 min skrócona o 50% daje opłatę 2 monet za pełne minuty, razem 167. Odrzucone paczki po 100 dałyby 252. Zakres czasu i zaokrąglenia pozostają założeniami.</t>
+        </is>
       </c>
     </row>
     <row r="8" customFormat="false" ht="114.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33760,8 +33912,10 @@
         <f aca="false">N8/Parametry!$C$41</f>
         <v>333.3</v>
       </c>
-      <c r="Q8" s="5" t="s">
-        <v>485</v>
+      <c r="Q8" s="5" t="inlineStr">
+        <is>
+          <t>Ratusz 1→2: portowa wartość materiałów 2250 ×1,25 = 2812,5; doliczamy osobno 500 monet. Przykładowa opłata czasowa 20 daje 3332,5; kalkulator roboczo zaokrągla do 3333. Samo końcowe zaokrąglenie nie jest jeszcze uzgodnione.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>